<commit_message>
correo.pty eliminado y unificado en registro.py
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1253,7 +1253,7 @@
           <t>fredy alexander calcetero pardo</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="2" t="n">
         <v>45889</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -1274,6 +1274,66 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>Con novedad</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>karen juliana cepeda garcia</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>45890</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sin novedad</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Tarde</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>karen juliana cepeda garcia</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>45890</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sin novedad</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Tarde</t>
         </is>
       </c>
     </row>

</xml_diff>